<commit_message>
Inward code fix and deployment setup
</commit_message>
<xml_diff>
--- a/NEW MASTER SHEET BILLING.xlsx
+++ b/NEW MASTER SHEET BILLING.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Carysil_Software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70E335F1-33A2-4C60-A091-C42637075CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34C565E-0F63-40F5-9FCE-8A8AEAC6CA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21486,10 +21486,10 @@
       </c>
       <c r="F24" s="109">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="105">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.4">

</xml_diff>